<commit_message>
claude tidy and jupyter file
</commit_message>
<xml_diff>
--- a/Missing_Event_Stream_Inserts.xlsx
+++ b/Missing_Event_Stream_Inserts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rapieruk-my.sharepoint.com/personal/ewan_hillnorris_rapieruk_com/Documents/Documents/GitHub/chillEpisodes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{08278EAB-B1FD-4E8D-A098-62D4DB43C1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="14_{08278EAB-B1FD-4E8D-A098-62D4DB43C1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDD0BFBA-294C-48A8-877A-FE1D562006E4}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Missing Inserts'!$A$1:$R$369</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3651" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3652" uniqueCount="750">
   <si>
     <t>Product</t>
   </si>
@@ -2289,6 +2288,9 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>HR1a,HR1b</t>
   </si>
 </sst>
 </file>
@@ -2991,7 +2993,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -3038,7 +3040,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -3124,7 +3126,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>18</v>
       </c>
@@ -3213,7 +3215,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>18</v>
       </c>
@@ -3256,7 +3258,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>18</v>
       </c>
@@ -3299,7 +3301,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
@@ -3342,7 +3344,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>18</v>
       </c>
@@ -3476,7 +3478,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>18</v>
       </c>
@@ -3519,7 +3521,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>18</v>
       </c>
@@ -3728,7 +3730,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>18</v>
       </c>
@@ -3771,7 +3773,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>18</v>
       </c>
@@ -3855,7 +3857,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>18</v>
       </c>
@@ -3896,7 +3898,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>18</v>
       </c>
@@ -3939,7 +3941,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>18</v>
       </c>
@@ -3973,7 +3975,7 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P29">
         <v>6836</v>
@@ -4025,7 +4027,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="31" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>18</v>
       </c>
@@ -4068,7 +4070,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>18</v>
       </c>
@@ -4152,7 +4154,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>18</v>
       </c>
@@ -4244,7 +4246,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>18</v>
       </c>
@@ -4289,7 +4291,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>18</v>
       </c>
@@ -4563,7 +4565,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>28</v>
       </c>
@@ -4739,7 +4741,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>28</v>
       </c>
@@ -4882,7 +4884,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="50" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>28</v>
       </c>
@@ -5201,7 +5203,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="57" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>28</v>
       </c>
@@ -5385,7 +5387,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="61" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>28</v>
       </c>
@@ -5428,7 +5430,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="62" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>28</v>
       </c>
@@ -5656,7 +5658,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="67" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
         <v>28</v>
       </c>
@@ -5699,7 +5701,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="68" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>28</v>
       </c>
@@ -5828,7 +5830,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="71" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
         <v>28</v>
       </c>
@@ -5871,7 +5873,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="72" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>28</v>
       </c>
@@ -5914,7 +5916,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="73" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>28</v>
       </c>
@@ -6123,7 +6125,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="78" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>28</v>
       </c>
@@ -6166,7 +6168,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>28</v>
       </c>
@@ -6211,7 +6213,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
         <v>28</v>
       </c>
@@ -6252,7 +6254,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
         <v>28</v>
       </c>
@@ -6294,7 +6296,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
         <v>28</v>
       </c>
@@ -6339,7 +6341,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
         <v>28</v>
       </c>
@@ -6384,7 +6386,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>28</v>
       </c>
@@ -6431,7 +6433,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
         <v>28</v>
       </c>
@@ -6519,7 +6521,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>28</v>
       </c>
@@ -6562,7 +6564,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="88" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>28</v>
       </c>
@@ -6605,7 +6607,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
         <v>28</v>
       </c>
@@ -6646,7 +6648,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
         <v>28</v>
       </c>
@@ -6687,7 +6689,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>28</v>
       </c>
@@ -6959,7 +6961,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="97" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>28</v>
       </c>
@@ -7002,7 +7004,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="98" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
         <v>28</v>
       </c>
@@ -7043,7 +7045,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="99" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
         <v>28</v>
       </c>
@@ -7451,7 +7453,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="108" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
         <v>28</v>
       </c>
@@ -7582,7 +7584,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="111" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
         <v>28</v>
       </c>
@@ -7623,7 +7625,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="112" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
         <v>28</v>
       </c>
@@ -7709,7 +7711,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="114" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>28</v>
       </c>
@@ -7886,7 +7888,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="118" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
         <v>28</v>
       </c>
@@ -7927,7 +7929,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="119" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
         <v>28</v>
       </c>
@@ -8051,13 +8053,16 @@
       <c r="M121" s="5"/>
       <c r="N121" s="5"/>
       <c r="O121" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="P121">
         <v>4396</v>
       </c>
       <c r="Q121" t="s">
-        <v>37</v>
+        <v>53</v>
+      </c>
+      <c r="R121" t="s">
+        <v>749</v>
       </c>
     </row>
     <row r="122" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
@@ -8107,7 +8112,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:18" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
         <v>28</v>
       </c>
@@ -8150,7 +8155,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="124" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
         <v>28</v>
       </c>
@@ -8554,7 +8559,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="133" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
         <v>28</v>
       </c>
@@ -8940,7 +8945,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="142" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
         <v>28</v>
       </c>
@@ -8981,7 +8986,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="143" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
         <v>28</v>
       </c>
@@ -9249,7 +9254,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="149" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A149" s="5" t="s">
         <v>28</v>
       </c>
@@ -9467,7 +9472,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="154" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A154" s="5" t="s">
         <v>28</v>
       </c>
@@ -9508,7 +9513,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="155" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A155" s="5" t="s">
         <v>28</v>
       </c>
@@ -9590,7 +9595,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="157" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A157" s="5" t="s">
         <v>28</v>
       </c>
@@ -9631,7 +9636,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="158" spans="1:18" ht="25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:18" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A158" s="5" t="s">
         <v>28</v>
       </c>
@@ -9803,7 +9808,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="162" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A162" s="5" t="s">
         <v>28</v>
       </c>
@@ -9844,7 +9849,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="163" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A163" s="5" t="s">
         <v>28</v>
       </c>
@@ -9929,7 +9934,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="165" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A165" s="5" t="s">
         <v>28</v>
       </c>
@@ -9970,7 +9975,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="166" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A166" s="5" t="s">
         <v>28</v>
       </c>
@@ -10011,7 +10016,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="167" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A167" s="5" t="s">
         <v>28</v>
       </c>
@@ -10093,7 +10098,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="169" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A169" s="5" t="s">
         <v>18</v>
       </c>
@@ -10134,7 +10139,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="170" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A170" s="5" t="s">
         <v>18</v>
       </c>
@@ -10175,7 +10180,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="171" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A171" s="5" t="s">
         <v>18</v>
       </c>
@@ -10216,7 +10221,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="172" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A172" s="5" t="s">
         <v>18</v>
       </c>
@@ -10257,7 +10262,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="173" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>18</v>
       </c>
@@ -10300,7 +10305,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="174" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A174" s="5" t="s">
         <v>18</v>
       </c>
@@ -10382,7 +10387,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="176" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A176" s="5" t="s">
         <v>18</v>
       </c>
@@ -10464,7 +10469,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="178" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A178" s="5" t="s">
         <v>18</v>
       </c>
@@ -10505,7 +10510,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="179" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A179" s="5" t="s">
         <v>18</v>
       </c>
@@ -10546,7 +10551,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="180" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>18</v>
       </c>
@@ -10589,7 +10594,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="181" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>18</v>
       </c>
@@ -10632,7 +10637,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="182" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>18</v>
       </c>
@@ -10675,7 +10680,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="183" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A183" s="5" t="s">
         <v>18</v>
       </c>
@@ -10718,7 +10723,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="184" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A184" s="5" t="s">
         <v>18</v>
       </c>
@@ -10761,7 +10766,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="185" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A185" s="5" t="s">
         <v>18</v>
       </c>
@@ -10804,7 +10809,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="186" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A186" s="5" t="s">
         <v>18</v>
       </c>
@@ -10847,7 +10852,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="187" spans="1:17" ht="25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:17" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" s="5" t="s">
         <v>18</v>
       </c>
@@ -11217,7 +11222,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="195" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A195" s="5" t="s">
         <v>18</v>
       </c>
@@ -11303,7 +11308,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="197" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A197" s="5" t="s">
         <v>18</v>
       </c>
@@ -11392,7 +11397,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="199" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A199" s="5" t="s">
         <v>18</v>
       </c>
@@ -11435,7 +11440,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="200" spans="1:18" ht="25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:18" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A200" s="5" t="s">
         <v>18</v>
       </c>
@@ -11524,7 +11529,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="202" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A202" s="5" t="s">
         <v>18</v>
       </c>
@@ -11567,7 +11572,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="203" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A203" s="5" t="s">
         <v>18</v>
       </c>
@@ -11610,7 +11615,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="204" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A204" s="5" t="s">
         <v>18</v>
       </c>
@@ -11657,7 +11662,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="205" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A205" s="5" t="s">
         <v>18</v>
       </c>
@@ -11788,7 +11793,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="208" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
         <v>25</v>
       </c>
@@ -11833,7 +11838,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="209" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>25</v>
       </c>
@@ -11878,7 +11883,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="210" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>25</v>
       </c>
@@ -11966,7 +11971,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="212" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A212" s="5" t="s">
         <v>445</v>
       </c>
@@ -12007,7 +12012,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="213" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
         <v>445</v>
       </c>
@@ -12096,7 +12101,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="215" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A215" s="5" t="s">
         <v>445</v>
       </c>
@@ -12137,7 +12142,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="216" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A216" s="5" t="s">
         <v>445</v>
       </c>
@@ -12178,7 +12183,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="217" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A217" s="5" t="s">
         <v>445</v>
       </c>
@@ -12219,7 +12224,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="218" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A218" s="5" t="s">
         <v>445</v>
       </c>
@@ -12305,7 +12310,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="220" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>445</v>
       </c>
@@ -12392,7 +12397,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="222" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A222" s="5" t="s">
         <v>445</v>
       </c>
@@ -12599,7 +12604,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="227" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A227" s="5" t="s">
         <v>445</v>
       </c>
@@ -12681,7 +12686,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="229" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>445</v>
       </c>
@@ -12724,7 +12729,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="230" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="2" t="s">
         <v>445</v>
       </c>
@@ -12808,7 +12813,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="232" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" s="5" t="s">
         <v>445</v>
       </c>
@@ -12849,7 +12854,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="233" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" s="5" t="s">
         <v>445</v>
       </c>
@@ -12890,7 +12895,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="234" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" s="2" t="s">
         <v>445</v>
       </c>
@@ -12933,7 +12938,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="235" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" s="5" t="s">
         <v>445</v>
       </c>
@@ -12965,7 +12970,7 @@
       <c r="M235" s="5"/>
       <c r="N235" s="5"/>
       <c r="O235" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P235">
         <v>8229</v>
@@ -13017,7 +13022,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="237" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A237" s="2" t="s">
         <v>445</v>
       </c>
@@ -13060,7 +13065,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="238" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A238" s="5" t="s">
         <v>445</v>
       </c>
@@ -13144,7 +13149,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="240" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A240" s="5" t="s">
         <v>445</v>
       </c>
@@ -13236,7 +13241,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="242" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A242" s="5" t="s">
         <v>445</v>
       </c>
@@ -13281,7 +13286,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="243" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A243" s="5" t="s">
         <v>445</v>
       </c>
@@ -13360,7 +13365,7 @@
       <c r="M244" s="2"/>
       <c r="N244" s="2"/>
       <c r="O244" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P244">
         <v>8203</v>
@@ -13401,7 +13406,7 @@
       <c r="M245" s="5"/>
       <c r="N245" s="5"/>
       <c r="O245" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P245">
         <v>8204</v>
@@ -13410,7 +13415,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="246" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A246" s="5" t="s">
         <v>445</v>
       </c>
@@ -13485,7 +13490,7 @@
       <c r="M247" s="2"/>
       <c r="N247" s="2"/>
       <c r="O247" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P247">
         <v>8206</v>
@@ -13570,7 +13575,7 @@
       <c r="M249" s="5"/>
       <c r="N249" s="5"/>
       <c r="O249" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P249">
         <v>8213</v>
@@ -13611,7 +13616,7 @@
       <c r="M250" s="5"/>
       <c r="N250" s="5"/>
       <c r="O250" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P250">
         <v>8216</v>
@@ -13652,7 +13657,7 @@
       <c r="M251" s="5"/>
       <c r="N251" s="5"/>
       <c r="O251" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P251">
         <v>8214</v>
@@ -13661,7 +13666,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="252" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A252" s="5" t="s">
         <v>445</v>
       </c>
@@ -13702,7 +13707,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="253" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A253" s="5" t="s">
         <v>445</v>
       </c>
@@ -13775,7 +13780,7 @@
       <c r="M254" s="5"/>
       <c r="N254" s="5"/>
       <c r="O254" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P254">
         <v>8208</v>
@@ -13816,7 +13821,7 @@
       <c r="M255" s="5"/>
       <c r="N255" s="5"/>
       <c r="O255" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P255">
         <v>8217</v>
@@ -13825,7 +13830,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="256" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A256" s="5" t="s">
         <v>445</v>
       </c>
@@ -13898,7 +13903,7 @@
       <c r="M257" s="5"/>
       <c r="N257" s="5"/>
       <c r="O257" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P257">
         <v>8210</v>
@@ -13953,7 +13958,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="259" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A259" s="5" t="s">
         <v>445</v>
       </c>
@@ -13994,7 +13999,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="260" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A260" s="5" t="s">
         <v>445</v>
       </c>
@@ -14035,7 +14040,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="261" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A261" s="5" t="s">
         <v>445</v>
       </c>
@@ -14076,7 +14081,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="262" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A262" s="5" t="s">
         <v>445</v>
       </c>
@@ -14117,7 +14122,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="263" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A263" s="5" t="s">
         <v>445</v>
       </c>
@@ -14158,7 +14163,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="264" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A264" s="2" t="s">
         <v>445</v>
       </c>
@@ -14340,7 +14345,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="268" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A268" s="5" t="s">
         <v>445</v>
       </c>
@@ -14381,7 +14386,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="269" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A269" s="5" t="s">
         <v>445</v>
       </c>
@@ -14565,7 +14570,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="273" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A273" s="5" t="s">
         <v>445</v>
       </c>
@@ -14606,7 +14611,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="274" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A274" s="2" t="s">
         <v>445</v>
       </c>
@@ -14685,7 +14690,7 @@
       <c r="M275" s="5"/>
       <c r="N275" s="5"/>
       <c r="O275" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P275">
         <v>7458</v>
@@ -14829,7 +14834,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="279" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A279" s="5" t="s">
         <v>445</v>
       </c>
@@ -14870,7 +14875,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="280" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A280" s="5" t="s">
         <v>445</v>
       </c>
@@ -17358,7 +17363,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="351" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
         <v>18</v>
       </c>
@@ -17901,7 +17906,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="366" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>445</v>
       </c>
@@ -18046,9 +18051,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R369" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
+    <filterColumn colId="14">
       <filters>
-        <filter val="Cancellation"/>
+        <filter val="empty"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>